<commit_message>
Update bedreflyt patient journey data to KG.xlsx
</commit_message>
<xml_diff>
--- a/ontology/background_documentation/bedreflyt patient journey data to KG.xlsx
+++ b/ontology/background_documentation/bedreflyt patient journey data to KG.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/laurasla/Documents/GitHub/bedreflyt/ontology/background_documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B062C1F-2080-244E-A8D6-F54281F0CA63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B4BB89-1F88-7647-BB44-2366037B22BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1740" yWindow="960" windowWidth="28160" windowHeight="17220" xr2:uid="{92AC32EE-E1DB-1542-A0D3-BC951B4FD252}"/>
+    <workbookView xWindow="11920" yWindow="1400" windowWidth="35300" windowHeight="22520" xr2:uid="{92AC32EE-E1DB-1542-A0D3-BC951B4FD252}"/>
   </bookViews>
   <sheets>
-    <sheet name="scenarios- simplified" sheetId="2" r:id="rId1"/>
-    <sheet name="scenarios- full" sheetId="1" r:id="rId2"/>
+    <sheet name="new scenarios simplified" sheetId="3" r:id="rId1"/>
+    <sheet name="scenarios- simplified" sheetId="2" r:id="rId2"/>
+    <sheet name="scenarios- full" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="155">
   <si>
     <t>Patient Diagnosis</t>
   </si>
@@ -211,6 +211,297 @@
   </si>
   <si>
     <t>1 hour ?</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>innkomst_I60</t>
+  </si>
+  <si>
+    <t>Subaraknoidal blodning innkomst I60</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I60_1</t>
+  </si>
+  <si>
+    <t>Subaraknoidal blodning observasjon I60</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I60_2</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I60_3</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I60_4</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I60_5</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I60_6</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I60_7</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I60_8</t>
+  </si>
+  <si>
+    <t>I601</t>
+  </si>
+  <si>
+    <t>innkomst_I601</t>
+  </si>
+  <si>
+    <t>Subaraknoidal blodning innkomst I601</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_1</t>
+  </si>
+  <si>
+    <t>Subaraknoidal blodning observasjon I601</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_2</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_3</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_4</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_5</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_6</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_7</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_8</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_9</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_10</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_11</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_12</t>
+  </si>
+  <si>
+    <t>observasjon_nev_I601_13</t>
+  </si>
+  <si>
+    <t>operasjon_M500</t>
+  </si>
+  <si>
+    <t>Lidelse i cervicalskive, med myelopati operasjon</t>
+  </si>
+  <si>
+    <t>sengeposten_M500</t>
+  </si>
+  <si>
+    <t>Lidelse i cervicalskive, med myelopati sengeposten</t>
+  </si>
+  <si>
+    <t>innkomst_G912</t>
+  </si>
+  <si>
+    <t>Normaltrykkshydrocephalus innkomst</t>
+  </si>
+  <si>
+    <t>operasjon_G912</t>
+  </si>
+  <si>
+    <t>Normaltrykkshydrocephalus operasjon</t>
+  </si>
+  <si>
+    <t>observasjon_G912</t>
+  </si>
+  <si>
+    <t>Normaltrykkshydrocephalus observasjon</t>
+  </si>
+  <si>
+    <t>S065</t>
+  </si>
+  <si>
+    <t>innkomst_S065</t>
+  </si>
+  <si>
+    <t>Kronisk subduralt hematom innkomst</t>
+  </si>
+  <si>
+    <t>operasjon_S065</t>
+  </si>
+  <si>
+    <t>Kronisk subduralt hematom operasjon</t>
+  </si>
+  <si>
+    <t>observasjon_S065</t>
+  </si>
+  <si>
+    <t>Kronisk subduralt hematom observasjon</t>
+  </si>
+  <si>
+    <t>D352</t>
+  </si>
+  <si>
+    <t>innkomst_D352</t>
+  </si>
+  <si>
+    <t>Hypofyseadenom innkomst</t>
+  </si>
+  <si>
+    <t>operasjon_D352</t>
+  </si>
+  <si>
+    <t>Hypofyseadenom operasjon</t>
+  </si>
+  <si>
+    <t>observasjon1_D352</t>
+  </si>
+  <si>
+    <t>Hypofyseadenom observasjon 1-2 timer</t>
+  </si>
+  <si>
+    <t>observasjon2_D352</t>
+  </si>
+  <si>
+    <t>Hypofyseadenom 24 timer</t>
+  </si>
+  <si>
+    <t>I671</t>
+  </si>
+  <si>
+    <t>innkomst_I671</t>
+  </si>
+  <si>
+    <t>Hjerneaneurisme uten ruptur innkomst</t>
+  </si>
+  <si>
+    <t>operasjon_I671</t>
+  </si>
+  <si>
+    <t>Hjerneaneurisme uten ruptur observasjon</t>
+  </si>
+  <si>
+    <t>observasjon1_I671</t>
+  </si>
+  <si>
+    <t>Hjerneaneurisme uten ruptur observasjon 1-2 timer</t>
+  </si>
+  <si>
+    <t>observasjon2_I671</t>
+  </si>
+  <si>
+    <t>Hjerneaneurisme uten ruptur</t>
+  </si>
+  <si>
+    <t>D320</t>
+  </si>
+  <si>
+    <t>innkomst_D320</t>
+  </si>
+  <si>
+    <t>Godartet svukst i hjernehinne innkomst</t>
+  </si>
+  <si>
+    <t>operasjon_D320</t>
+  </si>
+  <si>
+    <t>Godartet svukst i hjernehinne operasjon</t>
+  </si>
+  <si>
+    <t>observasjon_D320</t>
+  </si>
+  <si>
+    <t>Godartet svukst i hjernehinne observasjon</t>
+  </si>
+  <si>
+    <t>C712</t>
+  </si>
+  <si>
+    <t>innkomst_C712</t>
+  </si>
+  <si>
+    <t>Ondartet svulst i tinninglappen innkomst</t>
+  </si>
+  <si>
+    <t>operasjon_C712</t>
+  </si>
+  <si>
+    <t>Ondartet svulst i tinninglappen operasjon</t>
+  </si>
+  <si>
+    <t>observasjon_C712</t>
+  </si>
+  <si>
+    <t>Ondartet svulst i tinninglappen observasjon</t>
+  </si>
+  <si>
+    <t>M501</t>
+  </si>
+  <si>
+    <t>operasjon_M501</t>
+  </si>
+  <si>
+    <t>Lidelse i cervikalskrive, med radikulopati operasjon</t>
+  </si>
+  <si>
+    <t>observasjon_M501</t>
+  </si>
+  <si>
+    <t>Lidelse i cervikalskrive, med radikulopati observasjon</t>
+  </si>
+  <si>
+    <t>G500</t>
+  </si>
+  <si>
+    <t>innkomst_G500</t>
+  </si>
+  <si>
+    <t>Trigeminusnevralgi innkomst</t>
+  </si>
+  <si>
+    <t>operasjon_G500</t>
+  </si>
+  <si>
+    <t>Trigeminusnevralgi operasjon</t>
+  </si>
+  <si>
+    <t>observasjon_G500</t>
+  </si>
+  <si>
+    <t>Trigeminusnevralgi observasjon</t>
+  </si>
+  <si>
+    <t>C713</t>
+  </si>
+  <si>
+    <t>innkomst_C713</t>
+  </si>
+  <si>
+    <t>Ondartet svulst i isselapp innkomst</t>
+  </si>
+  <si>
+    <t>operasjon_C713</t>
+  </si>
+  <si>
+    <t>Ondartet svulst i isselapp intermediar</t>
+  </si>
+  <si>
+    <t>observasjon_C713</t>
+  </si>
+  <si>
+    <t>Ondartet svulst i isselapp observasjon</t>
   </si>
 </sst>
 </file>
@@ -252,9 +543,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,6 +880,1291 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{410655F7-8EA8-5047-AECF-5E18146AA313}">
+  <dimension ref="A1:G65"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2">
+        <v>2</v>
+      </c>
+      <c r="G3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="2">
+        <v>3</v>
+      </c>
+      <c r="G4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="2">
+        <v>4</v>
+      </c>
+      <c r="G5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="2">
+        <v>5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="2">
+        <v>6</v>
+      </c>
+      <c r="G7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C8">
+        <v>7</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2">
+        <v>7</v>
+      </c>
+      <c r="G8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" s="2">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="2">
+        <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B12" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="2">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="2">
+        <v>2</v>
+      </c>
+      <c r="G13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" s="2">
+        <v>3</v>
+      </c>
+      <c r="G14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="2">
+        <v>4</v>
+      </c>
+      <c r="G15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="2">
+        <v>5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17">
+        <v>6</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="2">
+        <v>6</v>
+      </c>
+      <c r="G17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18">
+        <v>7</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="2">
+        <v>7</v>
+      </c>
+      <c r="G18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19">
+        <v>8</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="2">
+        <v>8</v>
+      </c>
+      <c r="G19" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20">
+        <v>9</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" s="2">
+        <v>9</v>
+      </c>
+      <c r="G20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21">
+        <v>10</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" s="2">
+        <v>10</v>
+      </c>
+      <c r="G21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22">
+        <v>11</v>
+      </c>
+      <c r="D22">
+        <v>3</v>
+      </c>
+      <c r="E22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="2">
+        <v>11</v>
+      </c>
+      <c r="G22" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23">
+        <v>12</v>
+      </c>
+      <c r="D23">
+        <v>3</v>
+      </c>
+      <c r="E23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="2">
+        <v>12</v>
+      </c>
+      <c r="G23" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" t="s">
+        <v>85</v>
+      </c>
+      <c r="C24">
+        <v>13</v>
+      </c>
+      <c r="D24">
+        <v>3</v>
+      </c>
+      <c r="E24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" s="2">
+        <v>13</v>
+      </c>
+      <c r="G24" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25">
+        <v>14</v>
+      </c>
+      <c r="D25">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" s="2">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F26" s="2"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27">
+        <v>2</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27" t="s">
+        <v>38</v>
+      </c>
+      <c r="F27" s="2">
+        <v>1</v>
+      </c>
+      <c r="G27" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28">
+        <v>3</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28" t="s">
+        <v>25</v>
+      </c>
+      <c r="F28" s="2">
+        <v>2</v>
+      </c>
+      <c r="G28" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F29" s="2"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30" t="s">
+        <v>25</v>
+      </c>
+      <c r="F30" s="2">
+        <v>1</v>
+      </c>
+      <c r="G30" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31">
+        <v>2</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31" t="s">
+        <v>38</v>
+      </c>
+      <c r="F31" s="2">
+        <v>2</v>
+      </c>
+      <c r="G31" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>44</v>
+      </c>
+      <c r="B32" t="s">
+        <v>95</v>
+      </c>
+      <c r="C32">
+        <v>3</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32" t="s">
+        <v>25</v>
+      </c>
+      <c r="F32" s="2">
+        <v>3</v>
+      </c>
+      <c r="G32" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F33" s="2"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>97</v>
+      </c>
+      <c r="B34" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34">
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>2</v>
+      </c>
+      <c r="E34" t="s">
+        <v>38</v>
+      </c>
+      <c r="F34" s="2">
+        <v>1</v>
+      </c>
+      <c r="G34" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>97</v>
+      </c>
+      <c r="B35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C35">
+        <v>2</v>
+      </c>
+      <c r="D35">
+        <v>3</v>
+      </c>
+      <c r="E35" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" s="2">
+        <v>2</v>
+      </c>
+      <c r="G35" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>97</v>
+      </c>
+      <c r="B36" t="s">
+        <v>102</v>
+      </c>
+      <c r="C36">
+        <v>3</v>
+      </c>
+      <c r="D36">
+        <v>3</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" s="2">
+        <v>3</v>
+      </c>
+      <c r="G36" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" t="s">
+        <v>105</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38">
+        <v>2</v>
+      </c>
+      <c r="E38" t="s">
+        <v>38</v>
+      </c>
+      <c r="F38" s="2">
+        <v>1</v>
+      </c>
+      <c r="G38" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>104</v>
+      </c>
+      <c r="B39" t="s">
+        <v>107</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="D39">
+        <v>2</v>
+      </c>
+      <c r="E39" t="s">
+        <v>38</v>
+      </c>
+      <c r="F39" s="2">
+        <v>2</v>
+      </c>
+      <c r="G39" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>104</v>
+      </c>
+      <c r="B40" t="s">
+        <v>109</v>
+      </c>
+      <c r="C40">
+        <v>3</v>
+      </c>
+      <c r="D40">
+        <v>2</v>
+      </c>
+      <c r="E40" t="s">
+        <v>38</v>
+      </c>
+      <c r="F40" s="2">
+        <v>3</v>
+      </c>
+      <c r="G40" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>104</v>
+      </c>
+      <c r="B41" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41">
+        <v>4</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41" t="s">
+        <v>25</v>
+      </c>
+      <c r="F41" s="2">
+        <v>4</v>
+      </c>
+      <c r="G41" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F42" s="2"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>113</v>
+      </c>
+      <c r="B43" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="E43" t="s">
+        <v>25</v>
+      </c>
+      <c r="F43" s="2">
+        <v>1</v>
+      </c>
+      <c r="G43" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>113</v>
+      </c>
+      <c r="B44" t="s">
+        <v>116</v>
+      </c>
+      <c r="C44">
+        <v>2</v>
+      </c>
+      <c r="D44">
+        <v>2</v>
+      </c>
+      <c r="E44" t="s">
+        <v>38</v>
+      </c>
+      <c r="F44" s="2">
+        <v>2</v>
+      </c>
+      <c r="G44" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>113</v>
+      </c>
+      <c r="B45" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45">
+        <v>3</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45" t="s">
+        <v>25</v>
+      </c>
+      <c r="F45" s="2">
+        <v>3</v>
+      </c>
+      <c r="G45" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>113</v>
+      </c>
+      <c r="B46" t="s">
+        <v>120</v>
+      </c>
+      <c r="C46">
+        <v>4</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="E46" t="s">
+        <v>25</v>
+      </c>
+      <c r="F46" s="2">
+        <v>4</v>
+      </c>
+      <c r="G46" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F47" s="2"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>122</v>
+      </c>
+      <c r="B48" t="s">
+        <v>123</v>
+      </c>
+      <c r="C48">
+        <v>1</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48" t="s">
+        <v>38</v>
+      </c>
+      <c r="F48" s="2">
+        <v>1</v>
+      </c>
+      <c r="G48" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>122</v>
+      </c>
+      <c r="B49" t="s">
+        <v>125</v>
+      </c>
+      <c r="C49">
+        <v>2</v>
+      </c>
+      <c r="D49">
+        <v>2</v>
+      </c>
+      <c r="E49" t="s">
+        <v>38</v>
+      </c>
+      <c r="F49" s="2">
+        <v>2</v>
+      </c>
+      <c r="G49" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>122</v>
+      </c>
+      <c r="B50" t="s">
+        <v>127</v>
+      </c>
+      <c r="C50">
+        <v>3</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50" t="s">
+        <v>25</v>
+      </c>
+      <c r="F50" s="2">
+        <v>3</v>
+      </c>
+      <c r="G50" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F51" s="2"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>129</v>
+      </c>
+      <c r="B52" t="s">
+        <v>130</v>
+      </c>
+      <c r="C52">
+        <v>1</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52" t="s">
+        <v>25</v>
+      </c>
+      <c r="F52" s="2">
+        <v>1</v>
+      </c>
+      <c r="G52" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>129</v>
+      </c>
+      <c r="B53" t="s">
+        <v>132</v>
+      </c>
+      <c r="C53">
+        <v>2</v>
+      </c>
+      <c r="D53">
+        <v>2</v>
+      </c>
+      <c r="E53" t="s">
+        <v>38</v>
+      </c>
+      <c r="F53" s="2">
+        <v>2</v>
+      </c>
+      <c r="G53" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>129</v>
+      </c>
+      <c r="B54" t="s">
+        <v>134</v>
+      </c>
+      <c r="C54">
+        <v>3</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="E54" t="s">
+        <v>25</v>
+      </c>
+      <c r="F54" s="2">
+        <v>3</v>
+      </c>
+      <c r="G54" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F55" s="2"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>136</v>
+      </c>
+      <c r="B56" t="s">
+        <v>137</v>
+      </c>
+      <c r="C56">
+        <v>1</v>
+      </c>
+      <c r="D56">
+        <v>2</v>
+      </c>
+      <c r="E56" t="s">
+        <v>38</v>
+      </c>
+      <c r="F56" s="2">
+        <v>1</v>
+      </c>
+      <c r="G56" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>136</v>
+      </c>
+      <c r="B57" t="s">
+        <v>139</v>
+      </c>
+      <c r="C57">
+        <v>2</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="E57" t="s">
+        <v>25</v>
+      </c>
+      <c r="F57" s="2">
+        <v>2</v>
+      </c>
+      <c r="G57" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F58" s="2"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>141</v>
+      </c>
+      <c r="B59" t="s">
+        <v>142</v>
+      </c>
+      <c r="C59">
+        <v>1</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59" t="s">
+        <v>25</v>
+      </c>
+      <c r="F59" s="2">
+        <v>1</v>
+      </c>
+      <c r="G59" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>141</v>
+      </c>
+      <c r="B60" t="s">
+        <v>144</v>
+      </c>
+      <c r="C60">
+        <v>2</v>
+      </c>
+      <c r="D60">
+        <v>2</v>
+      </c>
+      <c r="E60" t="s">
+        <v>38</v>
+      </c>
+      <c r="F60" s="2">
+        <v>2</v>
+      </c>
+      <c r="G60" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>141</v>
+      </c>
+      <c r="B61" t="s">
+        <v>146</v>
+      </c>
+      <c r="C61">
+        <v>3</v>
+      </c>
+      <c r="D61">
+        <v>1</v>
+      </c>
+      <c r="E61" t="s">
+        <v>25</v>
+      </c>
+      <c r="F61" s="2">
+        <v>3</v>
+      </c>
+      <c r="G61" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F62" s="2"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>148</v>
+      </c>
+      <c r="B63" t="s">
+        <v>149</v>
+      </c>
+      <c r="C63">
+        <v>1</v>
+      </c>
+      <c r="D63">
+        <v>1</v>
+      </c>
+      <c r="E63" t="s">
+        <v>25</v>
+      </c>
+      <c r="F63" s="2">
+        <v>1</v>
+      </c>
+      <c r="G63" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>148</v>
+      </c>
+      <c r="B64" t="s">
+        <v>151</v>
+      </c>
+      <c r="C64">
+        <v>2</v>
+      </c>
+      <c r="D64">
+        <v>2</v>
+      </c>
+      <c r="E64" t="s">
+        <v>38</v>
+      </c>
+      <c r="F64" s="2">
+        <v>2</v>
+      </c>
+      <c r="G64" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>148</v>
+      </c>
+      <c r="B65" t="s">
+        <v>153</v>
+      </c>
+      <c r="C65">
+        <v>3</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+      <c r="E65" t="s">
+        <v>25</v>
+      </c>
+      <c r="F65" s="2">
+        <v>3</v>
+      </c>
+      <c r="G65" t="s">
+        <v>154</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE34CBD-467E-D140-83C0-59526FC94959}">
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -804,7 +2381,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDA4A77D-EC93-BE4C-994F-BA917D63C0AD}">
   <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>